<commit_message>
plate3d: roll the turret's barrel so the channel opens downward
The C section was lying on its side. A SECT runs along its plane's normal,
so the axis was already right and only the profile needed turning about it -
that is ROT.X here, not ROT.Z, which would have swung the length itself
round to +Y. Negative, so the mouth faces down as the drawing shows rather
than up.
</commit_message>
<xml_diff>
--- a/plate3d/PLATE3D_TURRET.xlsx
+++ b/plate3d/PLATE3D_TURRET.xlsx
@@ -1779,7 +1779,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>11</v>
       </c>
@@ -1806,6 +1806,9 @@
       </c>
       <c r="I46" t="s">
         <v>73</v>
+      </c>
+      <c r="J46">
+        <v>-90</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>